<commit_message>
Complete JKNG Automation till 05Mar26
</commit_message>
<xml_diff>
--- a/ExcelData/ExcelData.xlsx
+++ b/ExcelData/ExcelData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Credentials" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="87">
   <si>
     <t>URL</t>
   </si>
@@ -41,9 +41,6 @@
     <t>Split Qty</t>
   </si>
   <si>
-    <t>VKAUCT0405_000010-1</t>
-  </si>
-  <si>
     <t>TransporterName</t>
   </si>
   <si>
@@ -113,148 +110,178 @@
     <t>Vehicle Type</t>
   </si>
   <si>
+    <t>Driver License</t>
+  </si>
+  <si>
+    <t>Driver Name</t>
+  </si>
+  <si>
+    <t>Contact No</t>
+  </si>
+  <si>
+    <t>DLODR0001</t>
+  </si>
+  <si>
+    <t>License Expiry Date</t>
+  </si>
+  <si>
+    <t>OwnerShipType</t>
+  </si>
+  <si>
+    <t>Market</t>
+  </si>
+  <si>
+    <t>Engine No</t>
+  </si>
+  <si>
+    <t>Chassis No</t>
+  </si>
+  <si>
+    <t>Eng0001</t>
+  </si>
+  <si>
+    <t>Chs0001</t>
+  </si>
+  <si>
+    <t>RFIDMH02JP3875</t>
+  </si>
+  <si>
+    <t>Vinay Kadam</t>
+  </si>
+  <si>
+    <t>MH</t>
+  </si>
+  <si>
+    <t>Vehicle Capacity</t>
+  </si>
+  <si>
+    <t>TareWeight</t>
+  </si>
+  <si>
+    <t>GrossWeight</t>
+  </si>
+  <si>
+    <t>RC NO</t>
+  </si>
+  <si>
+    <t>RC0001</t>
+  </si>
+  <si>
+    <t>Manufacturing MonthYear</t>
+  </si>
+  <si>
+    <t>Manufacture By</t>
+  </si>
+  <si>
+    <t>India Asia</t>
+  </si>
+  <si>
+    <t>2022</t>
+  </si>
+  <si>
+    <t>February</t>
+  </si>
+  <si>
+    <t>Model NO</t>
+  </si>
+  <si>
+    <t>MOD0001</t>
+  </si>
+  <si>
+    <t>PUC Expiry Date</t>
+  </si>
+  <si>
+    <t>Road Tax Renew Date</t>
+  </si>
+  <si>
+    <t>Fitness Renew Date</t>
+  </si>
+  <si>
+    <t>Veh Registratnion date</t>
+  </si>
+  <si>
+    <t>Veh Expiry Date</t>
+  </si>
+  <si>
+    <t>Insurance No</t>
+  </si>
+  <si>
+    <t>INSIND001</t>
+  </si>
+  <si>
+    <t>Insurance Company</t>
+  </si>
+  <si>
+    <t>United India</t>
+  </si>
+  <si>
+    <t>Insurance Expiry Date</t>
+  </si>
+  <si>
+    <t>Leaveap@Feb26</t>
+  </si>
+  <si>
+    <t>Split Single order and Sent to Auction  to Single Transporter</t>
+  </si>
+  <si>
+    <t>PranjalTrans</t>
+  </si>
+  <si>
+    <t>VKAUCT0405_000010-79</t>
+  </si>
+  <si>
+    <t>PVC Issue Date</t>
+  </si>
+  <si>
+    <t>PVC Expiry Date</t>
+  </si>
+  <si>
+    <t>VK0OB30033_000010-1</t>
+  </si>
+  <si>
     <t>Truck</t>
   </si>
   <si>
-    <t>Driver License</t>
-  </si>
-  <si>
-    <t>Driver Name</t>
-  </si>
-  <si>
-    <t>Contact No</t>
-  </si>
-  <si>
-    <t>DLODR0001</t>
-  </si>
-  <si>
-    <t>License Expiry Date</t>
-  </si>
-  <si>
-    <t>OwnerShipType</t>
-  </si>
-  <si>
-    <t>Market</t>
-  </si>
-  <si>
-    <t>Engine No</t>
-  </si>
-  <si>
-    <t>Chassis No</t>
-  </si>
-  <si>
-    <t>Eng0001</t>
-  </si>
-  <si>
-    <t>Chs0001</t>
-  </si>
-  <si>
-    <t>RFIDMH02JP3875</t>
-  </si>
-  <si>
-    <t>Vinay Kadam</t>
-  </si>
-  <si>
-    <t>MH</t>
-  </si>
-  <si>
-    <t>Vehicle Capacity</t>
-  </si>
-  <si>
-    <t>TareWeight</t>
-  </si>
-  <si>
-    <t>GrossWeight</t>
-  </si>
-  <si>
-    <t>RC NO</t>
-  </si>
-  <si>
-    <t>RC0001</t>
-  </si>
-  <si>
-    <t>Manufacturing MonthYear</t>
-  </si>
-  <si>
-    <t>Manufacture By</t>
-  </si>
-  <si>
-    <t>India Asia</t>
-  </si>
-  <si>
-    <t>2022</t>
-  </si>
-  <si>
-    <t>February</t>
-  </si>
-  <si>
-    <t>Model NO</t>
-  </si>
-  <si>
-    <t>MOD0001</t>
-  </si>
-  <si>
-    <t>PUC Expiry Date</t>
-  </si>
-  <si>
-    <t>Road Tax Renew Date</t>
-  </si>
-  <si>
-    <t>Fitness Renew Date</t>
-  </si>
-  <si>
-    <t>Veh Registratnion date</t>
-  </si>
-  <si>
-    <t>Veh Expiry Date</t>
-  </si>
-  <si>
-    <t>Insurance No</t>
-  </si>
-  <si>
-    <t>INSIND001</t>
-  </si>
-  <si>
-    <t>Insurance Company</t>
-  </si>
-  <si>
-    <t>United India</t>
-  </si>
-  <si>
-    <t>Insurance Expiry Date</t>
-  </si>
-  <si>
-    <t>MH19114356</t>
-  </si>
-  <si>
-    <t>VKAUCT0405_000010-61</t>
-  </si>
-  <si>
-    <t>Leaveap@Feb26</t>
-  </si>
-  <si>
-    <t>MH22214554</t>
-  </si>
-  <si>
-    <t>VKAUCT0405_000010-66</t>
-  </si>
-  <si>
-    <t>MH22214843</t>
-  </si>
-  <si>
-    <t>VKAUCT0405_000010-67</t>
-  </si>
-  <si>
-    <t>MH22215919</t>
-  </si>
-  <si>
-    <t>VKAUCT0405_000010-68</t>
-  </si>
-  <si>
-    <t>MH22220923</t>
-  </si>
-  <si>
-    <t>VKAUCT0405_000010-69</t>
+    <t>MH09182217</t>
+  </si>
+  <si>
+    <t>VK0OB30033_000010-39</t>
+  </si>
+  <si>
+    <t>MH09182508</t>
+  </si>
+  <si>
+    <t>VK0OB30033_000010-40</t>
+  </si>
+  <si>
+    <t>MH17152604</t>
+  </si>
+  <si>
+    <t>VK0OB30033_000010-41</t>
+  </si>
+  <si>
+    <t>MH17153400</t>
+  </si>
+  <si>
+    <t>MH17153520</t>
+  </si>
+  <si>
+    <t>VK0OB30033_000010-42</t>
+  </si>
+  <si>
+    <t>MH17155726</t>
+  </si>
+  <si>
+    <t>MH17155834</t>
+  </si>
+  <si>
+    <t>VK0OB30033_000010-43</t>
+  </si>
+  <si>
+    <t>MH18160108</t>
+  </si>
+  <si>
+    <t>VK0OB30033_000010-44</t>
   </si>
 </sst>
 </file>
@@ -300,10 +327,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -600,16 +628,16 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s" s="0">
         <v>13</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="D1" t="s" s="0">
         <v>14</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="E1" t="s" s="0">
         <v>15</v>
-      </c>
-      <c r="E1" t="s" s="0">
-        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -620,13 +648,13 @@
         <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="D2" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -641,10 +669,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="47.85546875"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="54.7109375"/>
     <col min="2" max="2" bestFit="true" customWidth="true" width="21.140625"/>
     <col min="4" max="4" bestFit="true" customWidth="true" width="22.28515625"/>
     <col min="5" max="5" bestFit="true" customWidth="true" width="16.7109375"/>
@@ -655,7 +683,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s" s="0">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B1" t="s" s="0">
         <v>3</v>
@@ -667,52 +695,70 @@
         <v>4</v>
       </c>
       <c r="E1" t="s" s="0">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F1" t="s" s="0">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G1" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="H1" t="s" s="0">
         <v>19</v>
-      </c>
-      <c r="H1" t="s" s="0">
-        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s" s="0">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>6</v>
+        <v>71</v>
       </c>
       <c r="C2" s="0">
-        <v>2</v>
+        <v>2.77</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="E2" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="F2" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="F2" t="s" s="0">
-        <v>9</v>
-      </c>
       <c r="G2" t="s" s="0">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="H2" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="3"/>
+      <c r="E4" t="s" s="0">
+        <v>67</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:AD2"/>
+  <dimension ref="B1:AF2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" bestFit="true" customWidth="true" width="8.7109375"/>
@@ -742,119 +788,125 @@
     <col min="27" max="27" bestFit="true" customWidth="true" width="15.140625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:32" x14ac:dyDescent="0.25">
       <c r="B1" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="C1" t="s" s="0">
         <v>22</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="D1" t="s" s="0">
         <v>23</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="E1" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="F1" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="H1" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="I1" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="J1" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="K1" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="L1" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="M1" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="N1" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="O1" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="P1" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="Q1" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="R1" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="S1" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="T1" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="U1" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="V1" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="W1" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="X1" t="s" s="0">
+        <v>56</v>
+      </c>
+      <c r="Y1" t="s" s="0">
+        <v>57</v>
+      </c>
+      <c r="Z1" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="AA1" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="AB1" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="AC1" t="s" s="0">
+        <v>62</v>
+      </c>
+      <c r="AD1" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="AE1" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="AF1" t="s" s="0">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="2:32" x14ac:dyDescent="0.25">
+      <c r="B2" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="E2" t="s" s="0">
         <v>25</v>
       </c>
-      <c r="F1" t="s" s="0">
-        <v>27</v>
-      </c>
-      <c r="G1" t="s" s="0">
-        <v>29</v>
-      </c>
-      <c r="H1" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="I1" t="s" s="0">
+      <c r="F2" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="H2" t="s" s="0">
         <v>32</v>
       </c>
-      <c r="J1" t="s" s="0">
-        <v>33</v>
-      </c>
-      <c r="K1" t="s" s="0">
-        <v>35</v>
-      </c>
-      <c r="L1" t="s" s="0">
-        <v>36</v>
-      </c>
-      <c r="M1" t="s" s="0">
-        <v>38</v>
-      </c>
-      <c r="N1" t="s" s="0">
-        <v>39</v>
-      </c>
-      <c r="O1" t="s" s="0">
-        <v>45</v>
-      </c>
-      <c r="P1" t="s" s="0">
-        <v>46</v>
-      </c>
-      <c r="Q1" t="s" s="0">
-        <v>47</v>
-      </c>
-      <c r="R1" t="s" s="0">
-        <v>48</v>
-      </c>
-      <c r="S1" t="s" s="0">
-        <v>51</v>
-      </c>
-      <c r="T1" t="s" s="0">
-        <v>50</v>
-      </c>
-      <c r="U1" t="s" s="0">
-        <v>50</v>
-      </c>
-      <c r="V1" t="s" s="0">
-        <v>55</v>
-      </c>
-      <c r="W1" t="s" s="0">
-        <v>57</v>
-      </c>
-      <c r="X1" t="s" s="0">
-        <v>58</v>
-      </c>
-      <c r="Y1" t="s" s="0">
-        <v>59</v>
-      </c>
-      <c r="Z1" t="s" s="0">
-        <v>60</v>
-      </c>
-      <c r="AA1" t="s" s="0">
-        <v>61</v>
-      </c>
-      <c r="AB1" t="s" s="0">
-        <v>62</v>
-      </c>
-      <c r="AC1" t="s" s="0">
-        <v>64</v>
-      </c>
-      <c r="AD1" t="s" s="0">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="2" spans="2:30" x14ac:dyDescent="0.25">
-      <c r="B2" t="s" s="0">
-        <v>44</v>
-      </c>
-      <c r="C2" t="s" s="0">
-        <v>42</v>
-      </c>
-      <c r="D2" t="s" s="0">
-        <v>28</v>
-      </c>
-      <c r="E2" t="s" s="0">
-        <v>26</v>
-      </c>
-      <c r="F2" t="s" s="0">
-        <v>8</v>
-      </c>
-      <c r="G2" t="s" s="0">
-        <v>30</v>
-      </c>
-      <c r="H2" t="s" s="0">
-        <v>34</v>
-      </c>
       <c r="I2" t="s" s="0">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="J2" s="0">
         <v>9870580588</v>
@@ -863,13 +915,13 @@
         <v>26112030</v>
       </c>
       <c r="L2" t="s" s="0">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="M2" t="s" s="0">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="N2" t="s" s="0">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="O2" s="0">
         <v>99</v>
@@ -881,19 +933,19 @@
         <v>40</v>
       </c>
       <c r="R2" t="s" s="0">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="S2" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="T2" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="T2" s="2" t="s">
+      <c r="U2" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="V2" t="s" s="0">
         <v>54</v>
-      </c>
-      <c r="U2" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="V2" t="s" s="0">
-        <v>56</v>
       </c>
       <c r="W2" s="0">
         <v>23112030</v>
@@ -911,13 +963,19 @@
         <v>28112030</v>
       </c>
       <c r="AB2" t="s" s="0">
+        <v>61</v>
+      </c>
+      <c r="AC2" t="s" s="0">
         <v>63</v>
-      </c>
-      <c r="AC2" t="s" s="0">
-        <v>65</v>
       </c>
       <c r="AD2" s="0">
         <v>29112030</v>
+      </c>
+      <c r="AE2" s="0">
+        <v>23112025</v>
+      </c>
+      <c r="AF2" s="0">
+        <v>23112030</v>
       </c>
     </row>
   </sheetData>

</xml_diff>